<commit_message>
Extraindo Dados do site Magalu e exportando para um arquivo Excel usando as bibliotecas: Selenium, Pyautogui e Pandas
</commit_message>
<xml_diff>
--- a/Extraindo Dados Tabela (RPA)/Dados Extraidos/dadosAbasSite.xlsx
+++ b/Extraindo Dados Tabela (RPA)/Dados Extraidos/dadosAbasSite.xlsx
@@ -22,40 +22,40 @@
     <t># ID Due Date Invoice</t>
   </si>
   <si>
-    <t>1 j3v3f7e8zpb7teb9k3xtnv 28-06-2025</t>
-  </si>
-  <si>
-    <t>2 eqol3jshil9pfjzyj39l6 25-05-2025</t>
-  </si>
-  <si>
-    <t>3 ovxie42xw4mb8ywl404yxb 07-07-2025</t>
-  </si>
-  <si>
-    <t>4 2l1tunaxzapr04ze977nyr 09-09-2025</t>
-  </si>
-  <si>
-    <t>5 j1xojhzsfgq3h2m89mbu7b 19-09-2025</t>
-  </si>
-  <si>
-    <t>6 tjeht3g57p09w2037k9wo5 01-06-2025</t>
-  </si>
-  <si>
-    <t>7 0ji2082i7u24ormc76818x 05-08-2025</t>
-  </si>
-  <si>
-    <t>8 e6s3vle4cycimaeqeo4ia 14-07-2025</t>
-  </si>
-  <si>
-    <t>9 bt162p8iuqfq07ye7rzpmf 18-06-2025</t>
-  </si>
-  <si>
-    <t>10 368465ku0q49vw1ktl86ab 08-09-2025</t>
-  </si>
-  <si>
-    <t>11 9s58o7zpggs3m09d8epqq1 02-08-2025</t>
-  </si>
-  <si>
-    <t>12 mg3jlkdkukjdvmmhlx0mxb 28-08-2025</t>
+    <t>1 g39phlq9uyi9xoolx5jezd 18-06-2025</t>
+  </si>
+  <si>
+    <t>2 d27cxseja357ugwmbcghdv 06-07-2025</t>
+  </si>
+  <si>
+    <t>3 324o56y6isr9uz918biz5a 12-09-2025</t>
+  </si>
+  <si>
+    <t>4 sbh9s7othe8pe5jntzj1zi 18-06-2025</t>
+  </si>
+  <si>
+    <t>5 znmaqndwryof40hdy6ru46 06-07-2025</t>
+  </si>
+  <si>
+    <t>6 ejyf2odupd43ynbuinavb 28-07-2025</t>
+  </si>
+  <si>
+    <t>7 f4kbfl7twwp13ts8zcubtbi 04-08-2025</t>
+  </si>
+  <si>
+    <t>8 g1uv24nrhehcr4k1h1u3dm 19-07-2025</t>
+  </si>
+  <si>
+    <t>9 6xdsjt23ffppjcmz3vg4zg 09-09-2025</t>
+  </si>
+  <si>
+    <t>10 xwzxk18t7rpc286e6sb2n6 27-08-2025</t>
+  </si>
+  <si>
+    <t>11 hybjgz844m82cpbs82uvt7 15-07-2025</t>
+  </si>
+  <si>
+    <t>12 bz306hukp891x2yuhnfbg 09-08-2025</t>
   </si>
 </sst>
 </file>

</xml_diff>